<commit_message>
Updates for taxonomy and nomenclature
</commit_message>
<xml_diff>
--- a/galls_2026/DATA/Quercus_Hipp-et-al_metadata_2026-05-05.xlsx
+++ b/galls_2026/DATA/Quercus_Hipp-et-al_metadata_2026-05-05.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahipp\Dropbox\OAKS-MISC-PROJECTS\2024 - Reiss phylo\Kasey-phylo-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahipp\Documents\github\fagaceae-phylo\galls_2026\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBA0811-8C0F-471D-9000-5EF2D838DD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CC682A-525D-48A2-B98E-5FC80AE89E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{E9180B22-85F1-4113-85E8-89BA8011255A}"/>
   </bookViews>
@@ -28524,7 +28524,7 @@
         <v>201</v>
       </c>
       <c r="D248" s="2" t="s">
-        <v>3059</v>
+        <v>3058</v>
       </c>
       <c r="E248" s="9" t="s">
         <v>398</v>

</xml_diff>